<commit_message>
feat: adiciona plano de contas por cliente
</commit_message>
<xml_diff>
--- a/static/modelos/modelo_lancamentos_lote.xlsx
+++ b/static/modelos/modelo_lancamentos_lote.xlsx
@@ -425,8 +425,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="19" max="19"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -519,6 +522,11 @@
           <t>observacao</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>plano_de_contas</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -577,9 +585,6 @@
           <t>pix</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>350</v>
       </c>
@@ -588,7 +593,11 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>20.01</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -668,7 +677,11 @@
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>20.02</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>